<commit_message>
Fix summarization judge contract and remove undeclared Qwen Safety score
</commit_message>
<xml_diff>
--- a/tasks/summarization/ibm-granite-granite-4-2-8b/results.xlsx
+++ b/tasks/summarization/ibm-granite-granite-4-2-8b/results.xlsx
@@ -1,455 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Metrics" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Rubric" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sample" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Sample Rows" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Samples" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Judges" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Summary" sheetId="1" r:id="rId1"/>
+    <sheet name="Metrics" sheetId="2" r:id="rId2"/>
+    <sheet name="Rubric" sheetId="3" r:id="rId3"/>
+    <sheet name="Sample" sheetId="4" r:id="rId4"/>
+    <sheet name="Sample Rows" sheetId="5" r:id="rId5"/>
+    <sheet name="Samples" sheetId="6" r:id="rId6"/>
+    <sheet name="Judges" sheetId="7" r:id="rId7"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Metrics'!$A$1:$B$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Rubric'!$A$1:$F$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sample'!$A$1:$V$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sample Rows'!$A$1:$B$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Samples'!$A$1:$Q$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Judges'!$A$1:$I$7</definedName>
-  </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
-</file>
-
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
-    </font>
-  </fonts>
-  <fills count="3">
-    <fill>
-      <patternFill/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9EAF7"/>
-      </patternFill>
-    </fill>
-  </fills>
-  <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-  </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
-</styleSheet>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B35"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>field</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
@@ -554,325 +127,325 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>llm_judge_dimension_mean_0_to_5</t>
+          <t>llm_judge_faithfulness_pass_rate</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>4.94</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>huggingface_link</t>
+          <t>llm_judge_dimension_mean_0_to_5</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://huggingface.co/ibm-granite/granite-4.2-8b</t>
+          <t>4.94</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>model_description</t>
+          <t>huggingface_link</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>[](https://huggingface.co/collections/ibm-granite/granite-42-language-models) [](https://huggingface.co/blog/ibm-granite/granite-4-2) [](https://github.com/ibm-granite/granite-4.2-language-models) [](https://www.apache.org/licenses/LICENSE-2.0)</t>
+          <t>https://huggingface.co/ibm-granite/granite-4.2-8b</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>model_supported_languages</t>
+          <t>model_description</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>en, de, es, fr, ja, pt, ar, cs, it, ko, nl, zh</t>
+          <t>[](https://huggingface.co/collections/ibm-granite/granite-42-language-models) [](https://huggingface.co/blog/ibm-granite/granite-4-2) [](https://github.com/ibm-granite/granite-4.2-language-models) [](https://www.apache.org/licenses/LICENSE-2.0)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>eval_languages</t>
+          <t>model_supported_languages</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>en, de, es, fr, ja, pt, ar, cs, it, ko, nl, zh</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>assessment</t>
+          <t>eval_languages</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Judges found broadly acceptable outputs with no recurring edge case clearly isolated.</t>
+          <t>en</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>inference_time</t>
+          <t>assessment</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>16.275s p50 e2e @ c=1 (self_hosted_gpu_colab)</t>
+          <t>Judges found broadly acceptable outputs with no recurring edge case clearly isolated.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>hardware</t>
+          <t>inference_time</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>NVIDIA A100-SXM4-40GB (34.85 GB)</t>
+          <t>16.275s p50 e2e @ c=1 (self_hosted_gpu_colab)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>vllm_version</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0.30.0</t>
+          <t>NVIDIA A100-SXM4-40GB (34.85 GB)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>sample_source</t>
+          <t>vllm_version</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>combined</t>
+          <t>0.30.0</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>sample_sample_id</t>
+          <t>sample_source</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>c907fe7a8442</t>
+          <t>combined</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>sample_sample_count</t>
+          <t>sample_sample_id</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>c907fe7a8442</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>sample_jsonl</t>
+          <t>sample_sample_count</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>eval-runs/ibm-granite-granite-4-2-8b/summarization/standard/sample_combined_c907fe7a8442_n2.jsonl</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>sample_jsonl</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>eval-runs/ibm-granite-granite-4-2-8b/summarization/standard/sample_combined_c907fe7a8442_n2.jsonl</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>sample_dataset_count</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Definitions</t>
-        </is>
-      </c>
-    </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>term</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>meaning</t>
+          <t>Definitions</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>llm_judge_dimension_mean_0_to_5</t>
+          <t>term</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>For each sample, each valid LLM judge scores every graded rubric dimension from 0 to 5. The scorer averages judges per dimension, averages those graded dimensions into a sample score, then averages sample scores across the run. Binary gates such as Safety and Faithfulness are not included in this mean.</t>
+          <t>meaning</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>llm_judge_pass_rate</t>
+          <t>llm_judge_dimension_mean_0_to_5</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>The fraction of samples whose LLM-judge consensus passed: dimension mean is at least 3.0, no graded dimension is 0 or 1, and all binary/ranged gates pass.</t>
+          <t>For each sample, each valid LLM judge scores every graded rubric dimension from 0 to 5. The scorer averages judges per dimension, averages those graded dimensions into a sample score, then averages sample scores across the run. Binary gates such as Safety and Faithfulness are not included in this mean.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>model_supported_languages</t>
+          <t>llm_judge_pass_rate</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Languages claimed by the model card or model metadata. If the model card describes broad support without enumerating every language, the workbook keeps the concise claim, such as 'over 140 languages'.</t>
+          <t>The fraction of samples whose LLM-judge consensus passed: dimension mean is at least 3.0, no graded dimension is 0 or 1, and all binary/ranged gates pass.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>eval_languages</t>
+          <t>model_supported_languages</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Languages covered by this evaluation task or dataset. This is provenance for the run, not the full language capability of the model.</t>
+          <t>Languages claimed by the model card or model metadata. If the model card describes broad support without enumerating every language, the workbook keeps the concise claim, such as 'over 140 languages'.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>inference_time</t>
+          <t>eval_languages</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Performance headline latency. For remote third-party APIs this is the client-observed p50 end-to-end latency from the natural task run, normally at concurrency 1; it includes provider routing, queueing, network, image preprocessing, and model inference. For self-hosted Colab GPU runs it is GPU-only inference latency (no network/provider overhead).</t>
+          <t>Languages covered by this evaluation task or dataset. This is provenance for the run, not the full language capability of the model.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>hardware</t>
+          <t>inference_time</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>The hardware the performance timing was measured on. For self-hosted Colab runs this is the exact GPU (name and peak VRAM), pinned across models for comparability. For remote third-party APIs it records that the measurement was client-observed, since the serving hardware is not exposed.</t>
+          <t>Performance headline latency. For remote third-party APIs this is the client-observed p50 end-to-end latency from the natural task run, normally at concurrency 1; it includes provider routing, queueing, network, image preprocessing, and model inference. For self-hosted Colab GPU runs it is GPU-only inference latency (no network/provider overhead).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>vllm_version</t>
+          <t>hardware</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>The vLLM engine version that served a self-hosted Colab GPU performance run (the version actually imported on the VM, not merely the one requested). Recorded because the inference engine affects timing, so speed numbers are only comparable within one vLLM version. Absent for remote third-party API benchmarks, which do not use vLLM.</t>
+          <t>The hardware the performance timing was measured on. For self-hosted Colab runs this is the exact GPU (name and peak VRAM), pinned across models for comparability. For remote third-party APIs it records that the measurement was client-observed, since the serving hardware is not exposed.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>token_f1</t>
+          <t>vllm_version</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Token-level F1 between the model output and the reference: treats each as a bag of lowercased word tokens and computes the harmonic mean of precision (fraction of output tokens found in the reference) and recall (fraction of reference tokens found in the output). Ranges 0 to 1; order-insensitive, so it rewards content overlap rather than exact phrasing.</t>
+          <t>The vLLM engine version that served a self-hosted Colab GPU performance run (the version actually imported on the VM, not merely the one requested). Recorded because the inference engine affects timing, so speed numbers are only comparable within one vLLM version. Absent for remote third-party API benchmarks, which do not use vLLM.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>token_f1</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Token-level F1 between the model output and the reference: treats each as a bag of lowercased word tokens and computes the harmonic mean of precision (fraction of output tokens found in the reference) and recall (fraction of reference tokens found in the output). Ranges 0 to 1; order-insensitive, so it rewards content overlap rather than exact phrasing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>rouge_l</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>ROUGE-L F1 based on the longest common subsequence (LCS) between output and reference token sequences. Unlike token_f1 it respects word order (the LCS must appear in sequence), so it credits fluent, correctly-ordered overlap. Ranges 0 to 1.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B35"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>metric</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
@@ -995,55 +568,39 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B12"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>criterion</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>scale</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>score</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>meaning</t>
         </is>
@@ -1070,7 +627,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>misses nearly all key points or is off-topic.</t>
@@ -1098,7 +659,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>captures only a few peripheral points; most salient content is missing.</t>
@@ -1126,7 +691,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>captures some key points but omits several important ones or includes substantial irrelevant detail.</t>
@@ -1154,7 +723,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>captures the main points but with a notable omission or some irrelevant detail.</t>
@@ -1182,7 +755,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>captures most key points with only minor omissions.</t>
@@ -1210,7 +787,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>captures all salient points at an appropriate level of abstraction, closely matching the reference's coverage.</t>
@@ -1238,7 +819,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>disjointed, contradictory, or incoherent.</t>
@@ -1266,7 +851,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>barely organized; frequent jumps between ideas make it hard to follow.</t>
@@ -1294,7 +883,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>loosely organized; some ordering or logic problems.</t>
@@ -1322,7 +915,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>generally organized but with a noticeable ordering or transition problem.</t>
@@ -1350,7 +947,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>mostly well-organized with minor structural issues.</t>
@@ -1378,7 +979,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
           <t>clearly and logically organized; ideas flow naturally.</t>
@@ -1406,7 +1011,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
           <t>many fabricated or contradictory claims.</t>
@@ -1434,7 +1043,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>multiple fabricated or contradictory claims.</t>
@@ -1462,7 +1075,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
           <t>several unsupported claims.</t>
@@ -1490,7 +1107,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>mostly supported but with one clear unsupported claim.</t>
@@ -1518,7 +1139,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
           <t>largely faithful with a minor unsupported detail.</t>
@@ -1546,7 +1171,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
           <t>every claim is fully supported by the source.</t>
@@ -1574,7 +1203,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
           <t>severely ungrammatical or unreadable.</t>
@@ -1602,7 +1235,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F21" t="inlineStr">
         <is>
           <t>pervasive grammatical/word errors; often hard to read.</t>
@@ -1630,7 +1267,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F22" t="inlineStr">
         <is>
           <t>frequent grammatical/word errors that hinder reading.</t>
@@ -1658,7 +1299,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F23" t="inlineStr">
         <is>
           <t>several noticeable grammatical/word errors but still readable.</t>
@@ -1686,7 +1331,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F24" t="inlineStr">
         <is>
           <t>mostly fluent with minor errors.</t>
@@ -1714,7 +1363,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
           <t>fluent, polished, error-free prose.</t>
@@ -1742,7 +1395,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>contains clear hallucinations or fabricated facts.</t>
@@ -1770,7 +1427,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>mostly faithful but with a minor unsupported detail.</t>
@@ -1798,7 +1459,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
           <t>fully faithful; every statement is grounded in the source.</t>
@@ -1806,151 +1471,119 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F28"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:V8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="42" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="44" customWidth="1" min="14" max="14"/>
-    <col width="60" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="10" customWidth="1" min="20" max="20"/>
-    <col width="60" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>dataset_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>hf_id</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>source_hf_id</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>config</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>source_config</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>split</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>source_split</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>revision</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>source_revision</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>sample_count</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>sample_id</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>path</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>jsonl</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>default_input</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>row_count</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>hf_likes</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>license</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>paper</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>quality_evidence</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>reference_quality</t>
         </is>
@@ -1967,25 +1600,41 @@
           <t>local</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>ccdv/govreport-summarization</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>document</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>test</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
           <t>4e21184e01ae8017e2c036e180fe5e541fef60a0</t>
@@ -2016,7 +1665,11 @@
           <t>eval-runs/ibm-granite-granite-4-2-8b/summarization/standard/sample_local_1aab8ec6466f_n1_s1234.jsonl</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="Q2" t="inlineStr">
         <is>
           <t>1</t>
@@ -2032,7 +1685,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="U2" t="inlineStr">
         <is>
           <t>GovReport (Huang et al. 2021, arXiv:2104.02112) is a standard long-document summarization benchmark widely used in efficient-attention / long-context summarization papers and leaderboards. 973-row test split; report/summary fields with high-quality human reference summaries.</t>
@@ -2055,25 +1712,41 @@
           <t>local</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>FiscalNote/billsum</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>default</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>test</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>3d8510441c06a3d9dfb32eb0d7f80151730bcc4f</t>
@@ -2104,7 +1777,11 @@
           <t>eval-runs/ibm-granite-granite-4-2-8b/summarization/standard/sample_local_d2d408dbbd7c_n1_s1234.jsonl</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="Q3" t="inlineStr">
         <is>
           <t>1</t>
@@ -2120,7 +1797,11 @@
           <t>cc0-1.0</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="U3" t="inlineStr">
         <is>
           <t>BillSum (Kornilova &amp; Eidelman, ACL 2019 New Frontiers in Summarization, arXiv:1910.00523) is a well-established US-legislation summarization benchmark with human-written reference summaries; 3269-row test split.</t>
@@ -2177,31 +1858,19 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V8"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>dataset_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>row_index</t>
         </is>
@@ -2232,121 +1901,89 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B3"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Q3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="33" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="15" customWidth="1" min="14" max="14"/>
-    <col width="19" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="17" customWidth="1" min="17" max="17"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>dataset</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>input</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>reference</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>output</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>has_image</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>overall_pass</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>llm_judge_dimension_mean_0_to_5</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>safety_pass</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>faithfulness_pass</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>dim_Coherence</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>dim_Consistency</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>dim_Fluency</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>dim_Relevance</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>gate_Faithfulness</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>metric_rouge_l</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>metric_token_f1</t>
         </is>
@@ -2401,15 +2038,19 @@
           <t>4.88</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -2424,20 +2065,15 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>0.157</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
-        <is>
-          <t>0.157</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
         <is>
           <t>0.3916</t>
         </is>
@@ -2556,7 +2192,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Community Gardening and Nutrition Act of 2014 - Amends the Domestic Volunteer Service Act of 1973 to require the Director of the Corporation for National and Community Service to establish a Community Garden Pilot Program under the Volunteers in Service to America (VISTA) program. Requires the Program to address the health and nutrition of individuals in low-income and underserved communities through activities that include:  creating new community gardens and supporting and expanding existing community gardens; recruiting local community members to actively engage in community gardens and gardening projects; transforming vacant places into community garden plots; increasing community members' access to healthy foods and local foods while also encouraging them to stay active; expanding anti-poverty efforts by teaching basic nutrition and self-reliance through community gardening; and developing initiatives that increase the community's access to healthy, locally grown foods.  Requires the Director to carry out at least 40 projects under the Program. Requires the Director to give priority to: (1) volunteers with experience in health, nutrition, and gardening; (2) projects located in varied geographic regions; and (3) selecting a balance of urban and rural projects.  </t>
+          <t>Community Gardening and Nutrition Act of 2014 - Amends the Domestic Volunteer Service Act of 1973 to require the Director of the Corporation for National and Community Service to establish a Community Garden Pilot Program under the Volunteers in Service to America (VISTA) program. Requires the Program to address the health and nutrition of individuals in low-income and underserved communities through activities that include:  creating new community gardens and supporting and expanding existing community gardens; recruiting local community members to actively engage in community gardens and gardening projects; transforming vacant places into community garden plots; increasing community members' access to healthy foods and local foods while also encouraging them to stay active; expanding anti-poverty efforts by teaching basic nutrition and self-reliance through community gardening; and developing initiatives that increase the community's access to healthy, locally grown foods.  Requires the Director to carry out at least 40 projects under the Program. Requires the Director to give priority to: (1) volunteers with experience in health, nutrition, and gardening; (2) projects located in varied geographic regions; and (3) selecting a balance of urban and rural projects.  </t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -2595,10 +2231,14 @@
           <t>5.0</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -2618,93 +2258,69 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>0.1518</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>0.1518</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
           <t>0.33</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q3"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>sample_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>judge</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>parsed</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>reasoning</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Coherence</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Consistency</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Faithfulness</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Fluency</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Relevance</t>
         </is>
@@ -2820,12 +2436,36 @@
           <t>False</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2937,15 +2577,37 @@
           <t>False</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I7"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Remove Safety from the summarization evaluation contract
</commit_message>
<xml_diff>
--- a/tasks/summarization/ibm-granite-granite-4-2-8b/results.xlsx
+++ b/tasks/summarization/ibm-granite-granite-4-2-8b/results.xlsx
@@ -332,7 +332,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>For each sample, each valid LLM judge scores every graded rubric dimension from 0 to 5. The scorer averages judges per dimension, averages those graded dimensions into a sample score, then averages sample scores across the run. Binary gates such as Safety and Faithfulness are not included in this mean.</t>
+          <t>For each sample, each valid LLM judge scores every graded rubric dimension from 0 to 5. The scorer averages judges per dimension, averages those graded dimensions into a sample score, then averages sample scores across the run. Gate scores are not included in this mean.</t>
         </is>
       </c>
     </row>
@@ -527,7 +527,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>For each sample, each valid LLM judge scores every graded rubric dimension from 0 to 5. The scorer averages judges per dimension, averages those graded dimensions into a sample score, then averages sample scores across the run. Binary gates such as Safety and Faithfulness are not included in this mean.</t>
+          <t>For each sample, each valid LLM judge scores every graded rubric dimension from 0 to 5. The scorer averages judges per dimension, averages those graded dimensions into a sample score, then averages sample scores across the run. Gate scores are not included in this mean.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename LLM judge mean factor score across results and task views
</commit_message>
<xml_diff>
--- a/tasks/summarization/ibm-granite-granite-4-2-8b/results.xlsx
+++ b/tasks/summarization/ibm-granite-granite-4-2-8b/results.xlsx
@@ -439,7 +439,7 @@
   <dimension ref="A1:B53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -638,7 +638,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>llm_judge_dimension_mean_0_to_5</t>
+          <t>LLM Judge Mean Factor Score (0–5)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -910,7 +910,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>llm_judge_dimension_mean_0_to_5</t>
+          <t>LLM Judge Mean Factor Score (0–5)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1078,7 +1078,7 @@
   <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -1133,7 +1133,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>llm_judge_dimension_mean_0_to_5</t>
+          <t>LLM Judge Mean Factor Score (0–5)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1165,7 +1165,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>llm_judge_dimension_mean_0_to_5</t>
+          <t>LLM Judge Mean Factor Score (0–5)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2469,7 +2469,7 @@
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="33" customWidth="1" min="8" max="8"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
@@ -2518,7 +2518,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>llm_judge_dimension_mean_0_to_5</t>
+          <t>LLM Judge Mean Factor Score (0–5)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">

</xml_diff>